<commit_message>
İkinci inceleme: paylaşılabilir adresler, Genel Kurul görünümü, veri sözlüğü, yazım ve düzen
Özel depodaki c73bc9f'in yayın kopyası. Vetolar'da filtreler ve açık kayıt adreste, her kayda
bağlantı; "Genel Kurulda görüşülenler" görünümü; veto sayılmayan hayır oyları notu. Hakkında
beş bölüm, veri sözlüğü (CSV ve XLSX'lerde), gizlilik ve çevrimdışı sürüm satırları; sekme
sırası değişti; Metodoloji'de bölüm başlıkları 24 px. Barış gücü verisi 31 Temmuz 2026.
Görünen metinde kıvrık kesme, kurum adlarına gelen ekler kesmesiz (TDK), "evet, hayır,
çekimser". Hikâye adımları yayındaki hâlinde (üç düzeltmeyle). Sayılar aynı: 266 öneri,
322 ret oyu.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/veri/genel_kurul_tartismalari.xlsx
+++ b/web/veri/genel_kurul_tartismalari.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="genel_kurul_tartismalari" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sozluk" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'genel_kurul_tartismalari'!$A$1:$V$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'sozluk'!$A$1:$H$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -766,7 +768,7 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Toplantı kayıtları 30 Eylül 2022 vetosuna ve özel rapor A/77/551'e atıf yapıyor (A/ES-11/PV.12).</t>
+          <t>Toplantı kayıtları 30 Eylül 2022 vetosuna ve özel rapor A/77/551’e atıf yapıyor (A/ES-11/PV.12).</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1004,7 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>Toplantı kayıtlarında vetolara ve Konsey'in özel raporuna atıf var (A/ES-10/PV.40).</t>
+          <t>Toplantı kayıtlarında vetolara ve Konseyin özel raporuna atıf var (A/ES-10/PV.40).</t>
         </is>
       </c>
     </row>
@@ -2210,4 +2212,900 @@
   <autoFilter ref="A1:V22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dosya</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>sutun</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tip</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>bos_anlami</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>bos_anlami_en</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>degerler</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>aciklama_tr</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>aciklama_en</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>tartisma_id</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>metin</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tartışmanın kimliği. GK- önekinden sonra, olağanüstü özel oturumlarda oturumun adı (ES10, ES11), ardından ilk toplantı günü gelir.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Debate ID. The GK- prefix is followed by the emergency special session name where there is one (ES10, ES11), then by the first meeting day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>tur</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>kod</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>veto_girisimi | olaganustu_ozel_oturum</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Tartışmanın türü. veto_girisimi, vetodan sonra A/RES/76/262 uyarınca toplanan tartışmadır. olaganustu_ozel_oturum, Genel Kurulun aynı konuda olağanüstü özel oturumda toplandığını gösterir; bu durumda ayrı tartışma yapılmaz.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Type of debate. veto_girisimi is the debate convened after a veto under A/RES/76/262. olaganustu_ozel_oturum means the General Assembly met on the same matter in an emergency special session, in which case no separate debate is held.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>oturum</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>metin</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Genel Kurulun olağan oturum numarası ya da olağanüstü özel oturumun adı (ES-10, ES-11).</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Number of the regular General Assembly session, or the name of the emergency special session (ES-10, ES-11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>gundem_maddesi</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>metin</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Gündem maddesinin numarası ve BM'deki İngilizce başlığı.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Number of the agenda item and its UN title in English.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tarihler</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Tartışmanın toplantı günleri (YYYY-AA-GG).</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Meeting days of the debate (YYYY-MM-DD).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>toplanti_kayitlari</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Tartışmanın Genel Kurul toplantı kayıtları (A/…/PV.…).</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>General Assembly meeting records of the debate (A/…/PV.…).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>kayit_durumlari</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>resmi | gayriresmi_transkript | yayimlanmadi</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Her toplantı kaydının durumu, toplanti_kayitlari ile aynı sırada. resmi, tutanağın BM belge sisteminde yayımlandığını gösterir. gayriresmi_transkript, tutanak olmadığını ama BM'nin otomatik konuşma tanıma transkripti bulunduğunu gösterir. yayimlanmadi, ikisinin de olmadığını gösterir.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Status of each meeting record, in the same order as toplanti_kayitlari. resmi means the verbatim record is published in the UN document system. gayriresmi_transkript means there is no verbatim record yet but the UN's automatic speech-recognition transcript exists. yayimlanmadi means neither exists.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>veto_idleri</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Tartışmanın ele aldığı vetolar, vetolar.csv dosyasındaki id değerleriyle.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Vetoes covered by the debate, as id values from vetolar.csv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>aciklama_uye_devlet</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>tam sayı</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Veto gündem maddesinde açıklama yapan üye devlet sayısı. Her delegasyon bir kez sayılır, Başkan ve Sekretarya sayılmaz.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Number of Member States that made a statement under the veto agenda item. Each delegation counts once, and the President and the Secretariat are not counted. Empty for emergency special sessions, where speakers are not counted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>aciklama_gozlemci</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>tam sayı</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Açıklama yapan gözlemci sayısı. Avrupa Birliği ve Filistin Devleti gibi gözlemciler üye devletlerden ayrı sayılır.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Number of observers that made a statement. Observers such as the European Union and the State of Palestine are counted separately from Member States.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>gozlemciler</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Açıklama yapan gözlemcilerin BM'deki İngilizce adları.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Names of the observers that made a statement, as the UN writes them in English.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>grup_adina_konusan</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>tam sayı</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Açıklamasını bir grup adına yapan delegasyon sayısı. Her biri tek konuşmacı sayılır.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Number of delegations that spoke on behalf of a group. Each counts as one speaker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>grup_adina_konusanlar</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Grup adına konuşan delegasyonlar, Delegasyon (Grup) biçiminde.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Delegations that spoke on behalf of a group, in the form Delegation (Group).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>cevap_hakki</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>tam sayı</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Cevap hakkı kullanımlarının sayısı. Açıklamalardan ayrı tutulur.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Number of replies in exercise of the right of reply, counted separately from statements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>cevap_hakki_kullananlar</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum ya da cevap hakkı kullanılmadı</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Emergency special session, or the right of reply was not used</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Cevap hakkını kullanan delegasyonlar.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Delegations that exercised the right of reply. Empty when nobody did, or for emergency special sessions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>veto_eden_konustu</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>aciklama | yalnizca_cevap_hakki | hayir</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Veto eden her daimî üyenin tartışmada konuşup konuşmadığı, ÜYE:durum biçiminde (örnek: CHN:aciklama). aciklama, açıklama yaptığını; yalnizca_cevap_hakki, yalnızca cevap hakkını kullandığını gösterir. hayir, konuşmadığını gösterir.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Whether each vetoing permanent member spoke in the debate, in the form MEMBER:status (example: CHN:aciklama). aciklama means it made a statement, yalnizca_cevap_hakki that it spoke only in right of reply, and hayir that it did not speak.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>konusmaci_kaynagi</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>kod</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>toplanti_kaydi | bm_gunlugu | gayriresmi_transkript</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Konuşmacı sayımının kaynağı. toplanti_kaydi tutanaktır. bm_gunlugu, tutanak yayımlanmadığı için sayımın BM Günlüğü özetinden yapıldığını gösterir. gayriresmi_transkript, BM'nin otomatik transkriptidir.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Source of the speaker count. toplanti_kaydi is the verbatim record. bm_gunlugu means the count comes from the Journal of the United Nations summary because no verbatim record has been published. gayriresmi_transkript is the UN's automatic transcript.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>gayriresmi_alanlar</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Gayriresmî transkriptten alınmış bilgi yok</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No information taken from an informal transcript</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Gayriresmî transkriptten alınan bilgilerin işareti. Şu an bütün satırlarda boştur.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Marks information taken from an informal transcript. Empty in every row at present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>kabul_edilen_kararlar</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>liste (; ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Kayıtlı karar yok (veto girişimi tartışmaları)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No resolution recorded (veto initiative debates)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturumda kabul edilen Genel Kurul kararları (A/RES/…).</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>General Assembly resolutions adopted at the emergency special session (A/RES/…). Empty for veto initiative debates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>dogrulama</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>kod</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>dogrulandi | olasi</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Tartışmanın ilgili vetoyla bağının doğrulanma durumu. dogrulandi, tutanağın ya da BM Günlüğü'nün bu bağı gösterdiğini belirtir. olasi, bağın bu kaynaklardan kesinleşmediğini belirtir.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Whether the link between the debate and the veto is verified. dogrulandi means the verbatim record or the Journal of the United Nations shows the link. olasi means these sources do not settle it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>dogrulama_kaynagi</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>metin</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Boş olmaz</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Never empty</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Doğrulamanın dayanağı.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Basis for the verification, in Turkish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>genel_kurul_tartismalari.csv</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>capraz_kontrol</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>liste (| ile ayrılır)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Olağanüstü özel oturum; bu oturumlarda konuşmacı sayılmaz</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Emergency special session; speakers are not counted in these sessions</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Tutanaktan yapılan sayımın BM Günlüğü ve Başkanlık özetiyle karşılaştırması. Tutmayan her sayı yazılır.</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Comparison of the count with the Journal of the United Nations and the President's summary, in Turkish. Every mismatch is written down.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H23"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>